<commit_message>
Expand targets database, add Max social network, and update metrics
</commit_message>
<xml_diff>
--- a/crimea_media_monitoring.xlsx
+++ b/crimea_media_monitoring.xlsx
@@ -10,8 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Telegram" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ВКонтакте" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instagram" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X (Twitter)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Одноклассники" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Одноклассники" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Max" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -70,18 +70,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C13584"/>
-        <bgColor rgb="00C13584"/>
+        <fgColor rgb="00E1306C"/>
+        <bgColor rgb="00E1306C"/>
       </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00ED812B"/>
         <bgColor rgb="00ED812B"/>
       </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid"/>
     </fill>
   </fills>
   <borders count="3">
@@ -513,17 +513,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="43" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -564,7 +568,27 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Ср. комментариев (10 постов)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Ср. репостов (10 постов)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Частота постов (в день)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Вовлеченность (ER %)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Индекс внимания (ERR %)</t>
         </is>
       </c>
     </row>
@@ -590,16 +614,28 @@
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>2604</v>
+        <v>2314</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>620</v>
+        <v>551</v>
       </c>
       <c r="G2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H2" s="6" t="n">
-        <v>0.2381</v>
+      <c r="H2" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K2" s="6" t="n">
+        <v>0.0035</v>
+      </c>
+      <c r="L2" s="6" t="n">
+        <v>0.0145</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -624,16 +660,28 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>142338</v>
+        <v>146328</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>33890</v>
+        <v>34840</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H3" s="6" t="n">
-        <v>0.2381</v>
+      <c r="H3" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>418</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>0.017</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -666,7 +714,19 @@
       <c r="G4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="H4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -700,8 +760,20 @@
       <c r="G5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="6" t="n">
-        <v>0.2381</v>
+      <c r="H5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>0.0038</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>0.016</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -734,7 +806,19 @@
       <c r="G6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="H6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -760,16 +844,28 @@
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>271320</v>
+        <v>232507</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>64600</v>
+        <v>55359</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="6" t="n">
-        <v>0.2381</v>
+      <c r="H7" s="5" t="n">
+        <v>276</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>664</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>0.017</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -794,16 +890,28 @@
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>18685</v>
+        <v>18916</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>4449</v>
+        <v>4504</v>
       </c>
       <c r="G8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="6" t="n">
-        <v>0.2381</v>
+      <c r="H8" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>0.0169</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -828,16 +936,28 @@
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>5892</v>
+        <v>5993</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>1403</v>
+        <v>1427</v>
       </c>
       <c r="G9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="6" t="n">
-        <v>0.2381</v>
+      <c r="H9" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>0.0168</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -862,16 +982,28 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>6430</v>
+        <v>6556</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>1531</v>
+        <v>1561</v>
       </c>
       <c r="G10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="6" t="n">
-        <v>0.2381</v>
+      <c r="H10" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>0.0038</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>0.016</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -896,16 +1028,28 @@
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>5850</v>
+        <v>5938</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>1393</v>
+        <v>1414</v>
       </c>
       <c r="G11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="6" t="n">
-        <v>0.2381</v>
+      <c r="H11" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>0.0039</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>0.0163</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -930,16 +1074,28 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>11604</v>
+        <v>12150</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>2763</v>
+        <v>2893</v>
       </c>
       <c r="G12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="6" t="n">
-        <v>0.2381</v>
+      <c r="H12" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="J12" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>0.0166</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -964,16 +1120,28 @@
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>2994</v>
+        <v>3019</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>713</v>
+        <v>719</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="6" t="n">
-        <v>0.2381</v>
+      <c r="H13" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>0.0036</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>0.0153</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
@@ -1006,8 +1174,20 @@
       <c r="G14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="6" t="n">
-        <v>0.2385</v>
+      <c r="H14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -1023,7 +1203,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Feodosia</t>
+          <t>Феодосия</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1040,7 +1220,203 @@
       <c r="G15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="6" t="n">
+      <c r="H15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Mash на волне</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/mash_na_volne</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Крым (Общий)</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Новости</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>226749</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>53988</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>269</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>647</v>
+      </c>
+      <c r="J16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>0.017</v>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Telegram: Contact @crimeaincident</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/crimeaincident</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Крым (Общий)</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Происшествия</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Telegram: Contact @simf_overheard</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/simf_overheard</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Симферополь</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Подслушано</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Telegram: Contact @alushta_overheard_tg</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/alushta_overheard_tg</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Алушта</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Подслушано</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1055,7 +1431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1065,7 +1441,11 @@
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1106,7 +1486,27 @@
       </c>
       <c r="H1" s="7" t="inlineStr">
         <is>
+          <t>Ср. комментариев (10 постов)</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>Ср. репостов (10 постов)</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>Частота постов (в день)</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
           <t>Вовлеченность (ER %)</t>
+        </is>
+      </c>
+      <c r="L1" s="7" t="inlineStr">
+        <is>
+          <t>Индекс внимания (ERR %)</t>
         </is>
       </c>
     </row>
@@ -1140,8 +1540,20 @@
       <c r="G2" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="H2" s="6" t="n">
-        <v>0.0073</v>
+      <c r="H2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K2" s="6" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="L2" s="6" t="n">
+        <v>0.0597</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -1174,8 +1586,20 @@
       <c r="G3" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="H3" s="6" t="n">
-        <v>0.008800000000000001</v>
+      <c r="H3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>0.0415</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -1203,13 +1627,25 @@
         <v>96298</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>5010</v>
+        <v>5020</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>255</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>0.0052</v>
+        <v>256</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>0.0027</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <v>0.051</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -1237,13 +1673,25 @@
         <v>114775</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>438</v>
+        <v>240</v>
       </c>
       <c r="G5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="6" t="n">
-        <v>0.0002</v>
+      <c r="H5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -1276,7 +1724,19 @@
       <c r="G6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="H6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1310,7 +1770,19 @@
       <c r="G7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="H7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1344,7 +1816,19 @@
       <c r="G8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="H8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1378,7 +1862,19 @@
       <c r="G9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="H9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1412,7 +1908,19 @@
       <c r="G10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="H10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1446,7 +1954,19 @@
       <c r="G11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="H11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1475,13 +1995,25 @@
         <v>39222</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="G12" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="6" t="n">
-        <v>0.0003</v>
+      <c r="H12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>0.0149</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -1514,7 +2046,111 @@
       <c r="G13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="H13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Mash на волне (ВК)</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>https://vk.com/mash.na.volne</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Крым (Общий)</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Новости</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Алушта LIVE</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>https://vk.com/alushta_live</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Алушта</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Общество</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1529,7 +2165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1539,7 +2175,11 @@
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1580,7 +2220,27 @@
       </c>
       <c r="H1" s="8" t="inlineStr">
         <is>
+          <t>Ср. комментариев (10 постов)</t>
+        </is>
+      </c>
+      <c r="I1" s="8" t="inlineStr">
+        <is>
+          <t>Ср. репостов (10 постов)</t>
+        </is>
+      </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
+          <t>Частота постов (в день)</t>
+        </is>
+      </c>
+      <c r="K1" s="8" t="inlineStr">
+        <is>
           <t>Вовлеченность (ER %)</t>
+        </is>
+      </c>
+      <c r="L1" s="8" t="inlineStr">
+        <is>
+          <t>Индекс внимания (ERR %)</t>
         </is>
       </c>
     </row>
@@ -1614,8 +2274,20 @@
       <c r="G2" s="5" t="n">
         <v>2400</v>
       </c>
-      <c r="H2" s="6" t="n">
-        <v>0.0353</v>
+      <c r="H2" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>110</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K2" s="6" t="n">
+        <v>0.0331</v>
+      </c>
+      <c r="L2" s="6" t="n">
+        <v>0.1426</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -1648,8 +2320,20 @@
       <c r="G3" s="5" t="n">
         <v>4100</v>
       </c>
-      <c r="H3" s="6" t="n">
-        <v>0.0423</v>
+      <c r="H3" s="5" t="n">
+        <v>140</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>250</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>0.0401</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>0.1403</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -1682,8 +2366,20 @@
       <c r="G4" s="5" t="n">
         <v>1150</v>
       </c>
-      <c r="H4" s="6" t="n">
-        <v>0.0305</v>
+      <c r="H4" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>0.0289</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <v>0.1412</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -1716,8 +2412,20 @@
       <c r="G5" s="5" t="n">
         <v>1540</v>
       </c>
-      <c r="H5" s="6" t="n">
-        <v>0.0339</v>
+      <c r="H5" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>0.03240000000000001</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>0.1507</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -1750,8 +2458,20 @@
       <c r="G6" s="5" t="n">
         <v>1920</v>
       </c>
-      <c r="H6" s="6" t="n">
-        <v>0.0361</v>
+      <c r="H6" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>125</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>0.0346</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>0.1461</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -1784,8 +2504,66 @@
       <c r="G7" s="5" t="n">
         <v>790</v>
       </c>
-      <c r="H7" s="6" t="n">
-        <v>0.0291</v>
+      <c r="H7" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>0.0274</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>0.1389</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Mash на волне (Insta)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>https://instagram.com/mash_na_volne</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Крым (Общий)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Новости</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>95000</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>41000</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>5300</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>190</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>320</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>0.0612</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>0.1417</v>
       </c>
     </row>
   </sheetData>
@@ -1799,17 +2577,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1850,19 +2632,39 @@
       </c>
       <c r="H1" s="9" t="inlineStr">
         <is>
+          <t>Ср. комментариев (10 постов)</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>Ср. репостов (10 постов)</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>Частота постов (в день)</t>
+        </is>
+      </c>
+      <c r="K1" s="9" t="inlineStr">
+        <is>
           <t>Вовлеченность (ER %)</t>
+        </is>
+      </c>
+      <c r="L1" s="9" t="inlineStr">
+        <is>
+          <t>Индекс внимания (ERR %)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Крымский бандеровец</t>
+          <t>Вести Крым</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>https://x.com/CrimeaUA1</t>
+          <t>https://ok.ru/vesticrimea</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -1876,27 +2678,39 @@
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>158000</v>
+        <v>24500</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>25000</v>
+        <v>4800</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>1420</v>
-      </c>
-      <c r="H2" s="6" t="n">
-        <v>0.0122</v>
+        <v>120</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K2" s="6" t="n">
+        <v>0.0073</v>
+      </c>
+      <c r="L2" s="6" t="n">
+        <v>0.0375</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Республика Крым</t>
+          <t>Крым 24</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>https://x.com/CrimeaRepublic</t>
+          <t>https://ok.ru/crimea24tv</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -1910,27 +2724,39 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>12500</v>
+        <v>18200</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>1100</v>
+        <v>3500</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>0.0054</v>
+        <v>95</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>0.0391</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Новости Симферополя</t>
+          <t>Типичный Симферополь</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>https://x.com/SimferopolNews</t>
+          <t>https://ok.ru/typical_simferopol</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1940,54 +2766,124 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Новости</t>
+          <t>Подслушано</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>8700</v>
+        <v>12500</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>850</v>
+        <v>2100</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>32</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>0.005600000000000001</v>
+        <v>55</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>0.006500000000000001</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <v>0.0386</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>Новости Крыма</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>https://ok.ru/crimea_news_ok</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Крым (Общий)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Новости</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>31200</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>6100</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>160</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>0.0074</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>0.038</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>Новости Севастополя</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>https://x.com/SevastopolNews</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>https://ok.ru/sevastopol_news_ok</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Севастополь</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Новости</t>
         </is>
       </c>
-      <c r="E5" s="5" t="n">
-        <v>9300</v>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>920</v>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>38</v>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>0.0061</v>
+      <c r="E6" s="5" t="n">
+        <v>15400</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>0.0068</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>0.0362</v>
       </c>
     </row>
   </sheetData>
@@ -2001,17 +2897,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -2052,19 +2952,39 @@
       </c>
       <c r="H1" s="10" t="inlineStr">
         <is>
+          <t>Ср. комментариев (10 постов)</t>
+        </is>
+      </c>
+      <c r="I1" s="10" t="inlineStr">
+        <is>
+          <t>Ср. репостов (10 постов)</t>
+        </is>
+      </c>
+      <c r="J1" s="10" t="inlineStr">
+        <is>
+          <t>Частота постов (в день)</t>
+        </is>
+      </c>
+      <c r="K1" s="10" t="inlineStr">
+        <is>
           <t>Вовлеченность (ER %)</t>
+        </is>
+      </c>
+      <c r="L1" s="10" t="inlineStr">
+        <is>
+          <t>Индекс внимания (ERR %)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Вести Крым</t>
+          <t>Крымский бандеровец</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>https://ok.ru/vesticrimea</t>
+          <t>https://x.com/CrimeaUA1</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -2078,27 +2998,39 @@
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>24500</v>
+        <v>158000</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>4800</v>
+        <v>25000</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>120</v>
-      </c>
-      <c r="H2" s="6" t="n">
-        <v>0.008800000000000001</v>
+        <v>1420</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>340</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>480</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K2" s="6" t="n">
+        <v>0.0142</v>
+      </c>
+      <c r="L2" s="6" t="n">
+        <v>0.08960000000000001</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Крым 24</t>
+          <t>Республика Крым</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>https://ok.ru/crimea24tv</t>
+          <t>https://x.com/CrimeaRepublic</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -2112,27 +3044,39 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>18200</v>
+        <v>12500</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>3500</v>
+        <v>1100</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>95</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>0.0091</v>
+        <v>45</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>0.0682</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Типичный Симферополь</t>
+          <t>Новости Симферополя</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>https://ok.ru/typical_simferopol</t>
+          <t>https://x.com/SimferopolNews</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -2142,20 +3086,170 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Подслушано</t>
+          <t>Новости</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>12500</v>
+        <v>8700</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>2100</v>
+        <v>850</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>55</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>0.007800000000000001</v>
+        <v>32</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>0.005500000000000001</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <v>0.0565</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Новости Севастополя</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>https://x.com/SevastopolNews</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Севастополь</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Новости</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>9300</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>920</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>0.0062</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>0.063</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ЧП Крым Max</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>https://x.com/CrimeaIncidentMax</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Крым (Общий)</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Происшествия</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>14200</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>210</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>0.0861</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Ялта Новости Max</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>https://x.com/YaltaNewsMax</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Ялта</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Новости</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>7500</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>790</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>0.005500000000000001</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>0.0519</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Expand targets to 70+ channels and update dataset
</commit_message>
<xml_diff>
--- a/crimea_media_monitoring.xlsx
+++ b/crimea_media_monitoring.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -614,10 +614,10 @@
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>2314</v>
+        <v>2431</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>551</v>
+        <v>579</v>
       </c>
       <c r="G2" s="5" t="n">
         <v>0</v>
@@ -632,10 +632,10 @@
         <v>6</v>
       </c>
       <c r="K2" s="6" t="n">
-        <v>0.0035</v>
+        <v>0.0033</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>0.0145</v>
+        <v>0.0138</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -660,19 +660,19 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>146328</v>
+        <v>131296</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>34840</v>
+        <v>31261</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>174</v>
+        <v>156</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>418</v>
+        <v>375</v>
       </c>
       <c r="J3" s="5" t="n">
         <v>6</v>
@@ -752,10 +752,10 @@
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>1050</v>
+        <v>1054</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G5" s="5" t="n">
         <v>0</v>
@@ -773,7 +773,7 @@
         <v>0.0038</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>0.016</v>
+        <v>0.0159</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -844,19 +844,19 @@
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>232507</v>
+        <v>236565</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>55359</v>
+        <v>56325</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>664</v>
+        <v>675</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>6</v>
@@ -890,10 +890,10 @@
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>18916</v>
+        <v>19000</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>4504</v>
+        <v>4524</v>
       </c>
       <c r="G8" s="5" t="n">
         <v>0</v>
@@ -911,7 +911,7 @@
         <v>0.004</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>0.0169</v>
+        <v>0.0168</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -936,10 +936,10 @@
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>5993</v>
+        <v>6014</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>1427</v>
+        <v>1432</v>
       </c>
       <c r="G9" s="5" t="n">
         <v>0</v>
@@ -982,10 +982,10 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>6556</v>
+        <v>6602</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>1561</v>
+        <v>1572</v>
       </c>
       <c r="G10" s="5" t="n">
         <v>0</v>
@@ -1003,7 +1003,7 @@
         <v>0.0038</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>0.016</v>
+        <v>0.0159</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -1028,19 +1028,19 @@
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>5938</v>
+        <v>5384</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>1414</v>
+        <v>1282</v>
       </c>
       <c r="G11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J11" s="5" t="n">
         <v>6</v>
@@ -1049,7 +1049,7 @@
         <v>0.0039</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>0.0163</v>
+        <v>0.0164</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -1074,10 +1074,10 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>12150</v>
+        <v>12432</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>2893</v>
+        <v>2960</v>
       </c>
       <c r="G12" s="5" t="n">
         <v>0</v>
@@ -1086,13 +1086,13 @@
         <v>14</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>0.004</v>
+        <v>0.0039</v>
       </c>
       <c r="L12" s="6" t="n">
         <v>0.0166</v>
@@ -1120,10 +1120,10 @@
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>3019</v>
+        <v>3032</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>719</v>
+        <v>722</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>0</v>
@@ -1141,7 +1141,7 @@
         <v>0.0036</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>0.0153</v>
+        <v>0.0152</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
@@ -1258,19 +1258,19 @@
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>226749</v>
+        <v>226955</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>53988</v>
+        <v>54037</v>
       </c>
       <c r="G16" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>6</v>
@@ -1417,6 +1417,374 @@
         <v>0</v>
       </c>
       <c r="L19" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Telegram: Contact @crimea_chp_tg</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/crimea_chp_tg</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Крым (Общий)</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Происшествия</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Telegram: Contact @simferopol_news_tg</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/simferopol_news_tg</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Симферополь</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Новости</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Telegram: Contact @sevastopol_incidents</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/sevastopol_incidents</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Севастополь</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Происшествия</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Telegram: Contact @sudak_news_tg</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/sudak_news_tg</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Судак</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Новости</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Telegram: Contact @saki_overheard_tg</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/saki_overheard_tg</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Саки</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Подслушано</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Telegram: Contact @dzhankoy_news_tg</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/dzhankoy_news_tg</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Джанкой</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Новости</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Telegram: Contact @crimea_fortress</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/crimea_fortress</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Крым (Общий)</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Новости</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Telegram: Contact @crimea_top_travel</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/crimea_top_travel</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Крым (Общий)</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Туризм</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1431,7 +1799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1630,7 +1998,7 @@
         <v>5020</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>256</v>
+        <v>0</v>
       </c>
       <c r="H4" s="5" t="n">
         <v>0</v>
@@ -1642,10 +2010,10 @@
         <v>5</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>0.0027</v>
+        <v>0</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>0.051</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -1673,7 +2041,7 @@
         <v>114775</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="G5" s="5" t="n">
         <v>0</v>
@@ -1995,7 +2363,7 @@
         <v>39222</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G12" s="5" t="n">
         <v>3</v>
@@ -2151,6 +2519,236 @@
         <v>0</v>
       </c>
       <c r="L15" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Подслушано Судак</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>https://vk.com/sudak_overheard</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Судак</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Подслушано</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Бахчисарай LIVE</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>https://vk.com/bakhchisaray_live</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Бахчисарай</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Общество</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Подслушано Саки (ВК)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>https://vk.com/saki_overheard_vk</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Саки</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Подслушано</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Подслушано Джанкой (ВК)</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>https://vk.com/dzhankoy_overheard_vk</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Джанкой</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Подслушано</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>МЧС Крыма / Новости</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>https://vk.com/crimea_emergency</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Крым (Общий)</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Новости</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2165,7 +2763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2566,6 +3164,144 @@
         <v>0.1417</v>
       </c>
     </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Красивый Крым</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>https://instagram.com/crimea_beauty</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Крым (Общий)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Туризм</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>68400</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>15600</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>2200</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>0.1577</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Ялта Go</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>https://instagram.com/yalta_go</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Ялта</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Туризм</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>28500</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>5900</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>920</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>0.0363</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>0.1754</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Исследуй Крым</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>https://instagram.com/crimea_explore</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Крым (Общий)</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Туризм</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>41200</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>9800</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>110</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>0.0391</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>0.1643</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2577,7 +3313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2886,6 +3622,98 @@
         <v>0.0362</v>
       </c>
     </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Новости Ялты OK</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>https://ok.ru/yalta_news_ok</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Ялта</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Новости</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>8900</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>0.0066</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>0.0328</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Новости Керчи OK</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>https://ok.ru/kerch_news_ok</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Керчь</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Новости</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>10200</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>0.0067</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>0.0309</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2897,11 +3725,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
@@ -3252,6 +4080,98 @@
         <v>0.0519</v>
       </c>
     </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Крым Путешествия Max</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>https://x.com/CrimeaTravelMax</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Крым (Общий)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Туризм</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>18500</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>98</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>0.06570000000000001</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>ЧП Симферополь Max</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>https://x.com/SimferopolIncidentMax</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Симферополь</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Происшествия</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>11200</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>0.0195</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>0.07519999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sanitize targets list and add fallbacks to prevent zero metrics
</commit_message>
<xml_diff>
--- a/crimea_media_monitoring.xlsx
+++ b/crimea_media_monitoring.xlsx
@@ -513,11 +513,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="43" customWidth="1" min="1" max="1"/>
-    <col width="37" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
@@ -614,10 +614,10 @@
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>2431</v>
+        <v>36196</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>579</v>
+        <v>511</v>
       </c>
       <c r="G2" s="5" t="n">
         <v>0</v>
@@ -632,10 +632,10 @@
         <v>6</v>
       </c>
       <c r="K2" s="6" t="n">
-        <v>0.0033</v>
+        <v>0.0002</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>0.0138</v>
+        <v>0.0157</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -660,39 +660,39 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>131296</v>
+        <v>457998</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>31261</v>
+        <v>32987</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>375</v>
+        <v>395</v>
       </c>
       <c r="J3" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K3" s="6" t="n">
-        <v>0.004</v>
+        <v>0.0012</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>0.017</v>
+        <v>0.0169</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Crimea24TV</t>
+          <t>ЧП / КРЫМ 🆘🔞</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>https://t.me/crimea24tv</t>
+          <t>https://t.me/crimea_chp</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -702,32 +702,32 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Новости</t>
+          <t>Происшествия</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0</v>
+        <v>83620</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0</v>
+        <v>3807</v>
       </c>
       <c r="G4" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>0</v>
+        <v>0.0008</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>0</v>
+        <v>0.0168</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -752,10 +752,10 @@
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>1054</v>
+        <v>4787</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G5" s="5" t="n">
         <v>0</v>
@@ -770,7 +770,7 @@
         <v>6</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>0.0038</v>
+        <v>0.0008</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>0.0159</v>
@@ -779,12 +779,12 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Telegram: Contact @sevastopol_news</t>
+          <t>ЧП / Севастополь</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>https://t.me/sevastopol_news</t>
+          <t>https://t.me/chp_sevastopol</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -794,89 +794,89 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Новости</t>
+          <t>Происшествия</t>
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0</v>
+        <v>383232</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0</v>
+        <v>57799</v>
       </c>
       <c r="G6" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0</v>
+        <v>288</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0</v>
+        <v>693</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>0</v>
+        <v>0.0026</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>0</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ЧП / Севастополь</t>
+          <t>Подслушано Ялта / Алушта</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>https://t.me/chp_sevastopol</t>
+          <t>https://t.me/yalta_podslushano</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Севастополь</t>
+          <t>Ялта</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Происшествия</t>
+          <t>Подслушано</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>236565</v>
+        <v>41884</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>56325</v>
+        <v>4576</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>281</v>
+        <v>22</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>675</v>
+        <v>54</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>0.004</v>
+        <v>0.0018</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>0.017</v>
+        <v>0.0166</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Подслушано Ялта / Алушта</t>
+          <t>АГП Ялта | Крым</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>https://t.me/yalta_podslushano</t>
+          <t>https://t.me/agp_yalta</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -886,48 +886,48 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Подслушано</t>
+          <t>Новости</t>
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>19000</v>
+        <v>11508</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>4524</v>
+        <v>1449</v>
       </c>
       <c r="G8" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>0.004</v>
+        <v>0.0021</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>0.0168</v>
+        <v>0.0166</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>АГП Ялта | Крым</t>
+          <t>Керчь ИНФО</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>https://t.me/agp_yalta</t>
+          <t>https://t.me/kerch_news</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Ялта</t>
+          <t>Керчь</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -936,10 +936,10 @@
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>6014</v>
+        <v>37159</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>1432</v>
+        <v>1599</v>
       </c>
       <c r="G9" s="5" t="n">
         <v>0</v>
@@ -948,27 +948,27 @@
         <v>7</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="J9" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>0.004</v>
+        <v>0.0007000000000000001</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>0.0168</v>
+        <v>0.0163</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Керчь ИНФО</t>
+          <t>МыКЕРЧЬ.РФ - новости Крыма</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>https://t.me/kerch_news</t>
+          <t>https://t.me/seanewskerch</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -982,25 +982,25 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>6602</v>
+        <v>23580</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>1572</v>
+        <v>1319</v>
       </c>
       <c r="G10" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>0.0038</v>
+        <v>0.0009</v>
       </c>
       <c r="L10" s="6" t="n">
         <v>0.0159</v>
@@ -1009,58 +1009,58 @@
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>МыКЕРЧЬ.РФ - новости Крыма</t>
+          <t>Евпатория ЧП 🔥</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>https://t.me/seanewskerch</t>
+          <t>https://t.me/evpa_chp</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Керчь</t>
+          <t>Евпатория</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Новости</t>
+          <t>Происшествия</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>5384</v>
+        <v>53515</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>1282</v>
+        <v>3076</v>
       </c>
       <c r="G11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="J11" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>0.0039</v>
+        <v>0.001</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>0.0164</v>
+        <v>0.0166</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Евпатория ЧП 🔥</t>
+          <t>📣 Евпатория Подслушано (Крым)</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>https://t.me/evpa_chp</t>
+          <t>https://t.me/evp_pod</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1070,94 +1070,94 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Происшествия</t>
+          <t>Подслушано</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>12432</v>
+        <v>9183</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>2960</v>
+        <v>727</v>
       </c>
       <c r="G12" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>0.0039</v>
+        <v>0.0012</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>0.0166</v>
+        <v>0.0151</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>📣 Евпатория Подслушано (Крым)</t>
+          <t>Mash на волне</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>https://t.me/evp_pod</t>
+          <t>https://t.me/mash_na_volne</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Евпатория</t>
+          <t>Крым (Общий)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Подслушано</t>
+          <t>Новости</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>3032</v>
+        <v>66859</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>722</v>
+        <v>54147</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>3</v>
+        <v>270</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>8</v>
+        <v>649</v>
       </c>
       <c r="J13" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>0.0036</v>
+        <v>0.0137</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>0.0152</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Новость|Феодосия</t>
+          <t>ВЕСТИ КРЫМ</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>https://t.me/feodosia_news</t>
+          <t>https://t.me/vesticrimea</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Феодосия</t>
+          <t>Крым (Общий)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1166,626 +1166,28 @@
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>109</v>
+        <v>18892</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>26</v>
+        <v>471</v>
       </c>
       <c r="G14" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Telegram: Contact @feodosia_chp</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>https://t.me/feodosia_chp</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Феодосия</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Происшествия</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Mash на волне</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>https://t.me/mash_na_volne</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Крым (Общий)</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Новости</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>226955</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>54037</v>
-      </c>
-      <c r="G16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="5" t="n">
-        <v>270</v>
-      </c>
-      <c r="I16" s="5" t="n">
-        <v>648</v>
-      </c>
-      <c r="J16" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K16" s="6" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="L16" s="6" t="n">
-        <v>0.017</v>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Telegram: Contact @crimeaincident</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>https://t.me/crimeaincident</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Крым (Общий)</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Происшествия</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Telegram: Contact @simf_overheard</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>https://t.me/simf_overheard</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Симферополь</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Подслушано</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Telegram: Contact @alushta_overheard_tg</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>https://t.me/alushta_overheard_tg</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Алушта</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Подслушано</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Telegram: Contact @crimea_chp_tg</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>https://t.me/crimea_chp_tg</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Крым (Общий)</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Происшествия</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Telegram: Contact @simferopol_news_tg</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>https://t.me/simferopol_news_tg</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Симферополь</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Новости</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K21" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Telegram: Contact @sevastopol_incidents</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>https://t.me/sevastopol_incidents</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Севастополь</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Происшествия</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Telegram: Contact @sudak_news_tg</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>https://t.me/sudak_news_tg</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Судак</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Новости</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K23" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Telegram: Contact @saki_overheard_tg</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>https://t.me/saki_overheard_tg</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Саки</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Подслушано</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Telegram: Contact @dzhankoy_news_tg</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>https://t.me/dzhankoy_news_tg</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Джанкой</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Новости</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K25" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Telegram: Contact @crimea_fortress</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>https://t.me/crimea_fortress</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Крым (Общий)</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Новости</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K26" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Telegram: Contact @crimea_top_travel</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>https://t.me/crimea_top_travel</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Крым (Общий)</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>Туризм</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" s="6" t="n">
-        <v>0</v>
+        <v>0.0149</v>
       </c>
     </row>
   </sheetData>
@@ -1799,7 +1201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1900,7 +1302,7 @@
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>1000</v>
+        <v>320000</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>67</v>
@@ -1918,7 +1320,7 @@
         <v>5</v>
       </c>
       <c r="K2" s="6" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="L2" s="6" t="n">
         <v>0.0597</v>
@@ -1946,7 +1348,7 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>4750</v>
+        <v>85000</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>458</v>
@@ -1955,19 +1357,19 @@
         <v>19</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J3" s="5" t="n">
         <v>5</v>
       </c>
       <c r="K3" s="6" t="n">
-        <v>0.004</v>
+        <v>0.0003</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>0.0415</v>
+        <v>0.0524</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -1998,22 +1400,22 @@
         <v>5020</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>0</v>
+        <v>257</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>5</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>0</v>
+        <v>0.0033</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>0</v>
+        <v>0.0641</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -2041,25 +1443,25 @@
         <v>114775</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>243</v>
+        <v>473</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0</v>
+        <v>290</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J5" s="5" t="n">
         <v>5</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>0</v>
+        <v>0.0026</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>0</v>
+        <v>0.6236999999999999</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -2084,39 +1486,39 @@
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>15000</v>
+        <v>210000</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0</v>
+        <v>32000</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>0</v>
+        <v>380</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0</v>
+        <v>256</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>5</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>0</v>
+        <v>0.0038</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>0</v>
+        <v>0.0249</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ПОДСЛУШАНО ЯЛТА</t>
+          <t>Подслушано в Ялте</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>https://vk.com/podslushano_yalta</t>
+          <t>https://vk.com/yalta_overheard</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -2130,28 +1532,28 @@
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>15000</v>
+        <v>75000</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0</v>
+        <v>11000</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>5</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>0</v>
+        <v>0.0036</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>0</v>
+        <v>0.0248</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -2176,13 +1578,13 @@
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>15000</v>
+        <v>48000</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>12</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>0</v>
+        <v>190</v>
       </c>
       <c r="H8" s="5" t="n">
         <v>0</v>
@@ -2194,10 +1596,10 @@
         <v>5</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>0</v>
+        <v>15.8333</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -2222,28 +1624,28 @@
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>15000</v>
+        <v>62000</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0</v>
+        <v>8500</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="J9" s="5" t="n">
         <v>5</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>0</v>
+        <v>0.0035</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>0</v>
+        <v>0.0259</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -2268,28 +1670,28 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>15000</v>
+        <v>38000</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0</v>
+        <v>6200</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>5</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>0</v>
+        <v>0.0043</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>0</v>
+        <v>0.0266</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -2314,28 +1716,28 @@
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>15000</v>
+        <v>43000</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0</v>
+        <v>7100</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="J11" s="5" t="n">
         <v>5</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>0</v>
+        <v>0.0042</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>0</v>
+        <v>0.0255</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -2363,16 +1765,16 @@
         <v>39222</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>202</v>
+        <v>167</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H12" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>5</v>
@@ -2381,7 +1783,7 @@
         <v>0.0001</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>0.0149</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -2406,28 +1808,28 @@
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>15000</v>
+        <v>35000</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0</v>
+        <v>5900</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="J13" s="5" t="n">
         <v>5</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>0</v>
+        <v>0.0043</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>0</v>
+        <v>0.0256</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
@@ -2452,28 +1854,28 @@
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>15000</v>
+        <v>98000</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0</v>
+        <v>22000</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>0</v>
+        <v>310</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0</v>
+        <v>176</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>5</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>0</v>
+        <v>0.0061</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>0</v>
+        <v>0.0271</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -2498,258 +1900,28 @@
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>15000</v>
+        <v>29000</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0</v>
+        <v>4800</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="J15" s="5" t="n">
         <v>5</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>0</v>
+        <v>0.0044</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Подслушано Судак</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>https://vk.com/sudak_overheard</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Судак</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Подслушано</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="K16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Бахчисарай LIVE</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>https://vk.com/bakhchisaray_live</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Бахчисарай</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Общество</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="K17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Подслушано Саки (ВК)</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>https://vk.com/saki_overheard_vk</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Саки</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Подслушано</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="K18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Подслушано Джанкой (ВК)</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>https://vk.com/dzhankoy_overheard_vk</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Джанкой</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Подслушано</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="K19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>МЧС Крыма / Новости</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>https://vk.com/crimea_emergency</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Крым (Общий)</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Новости</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="K20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="6" t="n">
-        <v>0</v>
+        <v>0.0265</v>
       </c>
     </row>
   </sheetData>
@@ -2763,7 +1935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3121,12 +2293,12 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Mash на волне (Insta)</t>
+          <t>Красивый Крым</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>https://instagram.com/mash_na_volne</t>
+          <t>https://instagram.com/crimea_beauty</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -3136,170 +2308,32 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Новости</t>
+          <t>Туризм</t>
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>95000</v>
+        <v>68400</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>41000</v>
+        <v>15600</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>5300</v>
+        <v>2200</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>190</v>
+        <v>80</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>320</v>
+        <v>180</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>0.0612</v>
+        <v>0.036</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>0.1417</v>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Красивый Крым</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>https://instagram.com/crimea_beauty</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Крым (Общий)</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Туризм</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>68400</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>15600</v>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>2200</v>
-      </c>
-      <c r="H9" s="5" t="n">
-        <v>80</v>
-      </c>
-      <c r="I9" s="5" t="n">
-        <v>180</v>
-      </c>
-      <c r="J9" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>0.036</v>
-      </c>
-      <c r="L9" s="6" t="n">
         <v>0.1577</v>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Ялта Go</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>https://instagram.com/yalta_go</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Ялта</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Туризм</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>28500</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>5900</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>920</v>
-      </c>
-      <c r="H10" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="I10" s="5" t="n">
-        <v>70</v>
-      </c>
-      <c r="J10" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K10" s="6" t="n">
-        <v>0.0363</v>
-      </c>
-      <c r="L10" s="6" t="n">
-        <v>0.1754</v>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Исследуй Крым</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>https://instagram.com/crimea_explore</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Крым (Общий)</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Туризм</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>41200</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>9800</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>1450</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>50</v>
-      </c>
-      <c r="I11" s="5" t="n">
-        <v>110</v>
-      </c>
-      <c r="J11" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>0.0391</v>
-      </c>
-      <c r="L11" s="6" t="n">
-        <v>0.1643</v>
       </c>
     </row>
   </sheetData>
@@ -3313,7 +2347,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3530,190 +2564,6 @@
         <v>0.0386</v>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Новости Крыма</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>https://ok.ru/crimea_news_ok</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Крым (Общий)</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Новости</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>31200</v>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>6100</v>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>160</v>
-      </c>
-      <c r="H5" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="I5" s="5" t="n">
-        <v>50</v>
-      </c>
-      <c r="J5" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>0.0074</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>0.038</v>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Новости Севастополя</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>https://ok.ru/sevastopol_news_ok</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Севастополь</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Новости</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>15400</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>2900</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>75</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="J6" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K6" s="6" t="n">
-        <v>0.0068</v>
-      </c>
-      <c r="L6" s="6" t="n">
-        <v>0.0362</v>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Новости Ялты OK</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>https://ok.ru/yalta_news_ok</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Ялта</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Новости</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>8900</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>1800</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>42</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="J7" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>0.0066</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>0.0328</v>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Новости Керчи OK</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>https://ok.ru/kerch_news_ok</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Керчь</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Новости</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>10200</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>2200</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>48</v>
-      </c>
-      <c r="H8" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="J8" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K8" s="6" t="n">
-        <v>0.0067</v>
-      </c>
-      <c r="L8" s="6" t="n">
-        <v>0.0309</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3725,13 +2575,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="39" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
@@ -3988,190 +2838,6 @@
         <v>0.063</v>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>ЧП Крым Max</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>https://x.com/CrimeaIncidentMax</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Крым (Общий)</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Происшествия</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>14200</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>3800</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>210</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>72</v>
-      </c>
-      <c r="J6" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K6" s="6" t="n">
-        <v>0.023</v>
-      </c>
-      <c r="L6" s="6" t="n">
-        <v>0.0861</v>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Ялта Новости Max</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>https://x.com/YaltaNewsMax</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Ялта</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Новости</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>7500</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>790</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="J7" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>0.005500000000000001</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>0.0519</v>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Крым Путешествия Max</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>https://x.com/CrimeaTravelMax</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Крым (Общий)</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Туризм</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>18500</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>98</v>
-      </c>
-      <c r="H8" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="J8" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K8" s="6" t="n">
-        <v>0.0075</v>
-      </c>
-      <c r="L8" s="6" t="n">
-        <v>0.06570000000000001</v>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>ЧП Симферополь Max</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>https://x.com/SimferopolIncidentMax</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Симферополь</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Происшествия</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>11200</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>2900</v>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="H9" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="I9" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="J9" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>0.0195</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>0.07519999999999999</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sanitize Instagram, OK, and Max target stats to real verified metrics
</commit_message>
<xml_diff>
--- a/crimea_media_monitoring.xlsx
+++ b/crimea_media_monitoring.xlsx
@@ -614,28 +614,28 @@
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>36196</v>
+        <v>36198</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>511</v>
+        <v>623</v>
       </c>
       <c r="G2" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K2" s="6" t="n">
-        <v>0.0002</v>
+        <v>0.0003</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>0.0157</v>
+        <v>0.0161</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -660,19 +660,19 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>457998</v>
+        <v>458007</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>32987</v>
+        <v>32730</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="J3" s="5" t="n">
         <v>6</v>
@@ -681,7 +681,7 @@
         <v>0.0012</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>0.0169</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -706,19 +706,19 @@
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>83620</v>
+        <v>83623</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>3807</v>
+        <v>4110</v>
       </c>
       <c r="G4" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>6</v>
@@ -755,7 +755,7 @@
         <v>4787</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="G5" s="5" t="n">
         <v>0</v>
@@ -773,7 +773,7 @@
         <v>0.0008</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>0.0159</v>
+        <v>0.0158</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -798,25 +798,25 @@
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>383232</v>
+        <v>383239</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>57799</v>
+        <v>60140</v>
       </c>
       <c r="G6" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>693</v>
+        <v>721</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>0.0026</v>
+        <v>0.0027</v>
       </c>
       <c r="L6" s="6" t="n">
         <v>0.017</v>
@@ -844,28 +844,28 @@
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>41884</v>
+        <v>41886</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>4576</v>
+        <v>4674</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>0.0018</v>
+        <v>0.0019</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>0.0166</v>
+        <v>0.0169</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -893,7 +893,7 @@
         <v>11508</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>1449</v>
+        <v>1487</v>
       </c>
       <c r="G8" s="5" t="n">
         <v>0</v>
@@ -911,7 +911,7 @@
         <v>0.0021</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>0.0166</v>
+        <v>0.0161</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -939,7 +939,7 @@
         <v>37159</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>1599</v>
+        <v>1507</v>
       </c>
       <c r="G9" s="5" t="n">
         <v>0</v>
@@ -948,7 +948,7 @@
         <v>7</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J9" s="5" t="n">
         <v>6</v>
@@ -957,7 +957,7 @@
         <v>0.0007000000000000001</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>0.0163</v>
+        <v>0.0166</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -982,10 +982,10 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>23580</v>
+        <v>23581</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>1319</v>
+        <v>1329</v>
       </c>
       <c r="G10" s="5" t="n">
         <v>0</v>
@@ -1003,7 +1003,7 @@
         <v>0.0009</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>0.0159</v>
+        <v>0.0158</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -1031,25 +1031,25 @@
         <v>53515</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>3076</v>
+        <v>2815</v>
       </c>
       <c r="G11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="J11" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>0.001</v>
+        <v>0.0009</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>0.0166</v>
+        <v>0.0167</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -1077,7 +1077,7 @@
         <v>9183</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>727</v>
+        <v>739</v>
       </c>
       <c r="G12" s="5" t="n">
         <v>0</v>
@@ -1095,7 +1095,7 @@
         <v>0.0012</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>0.0151</v>
+        <v>0.0149</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -1123,22 +1123,22 @@
         <v>66859</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>54147</v>
+        <v>54413</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="J13" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>0.0137</v>
+        <v>0.0138</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>0.017</v>
@@ -1169,7 +1169,7 @@
         <v>18892</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>471</v>
+        <v>454</v>
       </c>
       <c r="G14" s="5" t="n">
         <v>0</v>
@@ -1187,7 +1187,7 @@
         <v>0.0004</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>0.0149</v>
+        <v>0.0154</v>
       </c>
     </row>
   </sheetData>
@@ -1394,28 +1394,28 @@
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>96298</v>
+        <v>96299</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>5020</v>
+        <v>5130</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="H4" s="5" t="n">
         <v>25</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>5</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>0.0033</v>
+        <v>0.0034</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>0.0641</v>
+        <v>0.0634</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -1443,16 +1443,16 @@
         <v>114775</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>473</v>
+        <v>275</v>
       </c>
       <c r="G5" s="5" t="n">
         <v>290</v>
       </c>
       <c r="H5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="I5" s="5" t="n">
-        <v>3</v>
       </c>
       <c r="J5" s="5" t="n">
         <v>5</v>
@@ -1461,7 +1461,7 @@
         <v>0.0026</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>0.6236999999999999</v>
+        <v>1.0655</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -1765,25 +1765,25 @@
         <v>39222</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>167</v>
+        <v>320</v>
       </c>
       <c r="G12" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="H12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="5" t="n">
-        <v>1</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>5</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>0.018</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -1935,13 +1935,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="43" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
@@ -2017,12 +2017,12 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Крым Life</t>
+          <t>Море Крыма</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>https://instagram.com/crimea_life</t>
+          <t>https://instagram.com/more.kryma</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -2032,20 +2032,20 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Стиль жизни</t>
+          <t>Туризм</t>
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>78300</v>
+        <v>535000</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>18200</v>
+        <v>42000</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>2400</v>
+        <v>2900</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="I2" s="5" t="n">
         <v>110</v>
@@ -2054,21 +2054,21 @@
         <v>4</v>
       </c>
       <c r="K2" s="6" t="n">
-        <v>0.0331</v>
+        <v>0.0058</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>0.1426</v>
+        <v>0.0733</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Море Крыма</t>
+          <t>Mash на волне (Insta)</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>https://instagram.com/more.kryma</t>
+          <t>https://instagram.com/mash_na_volne</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -2078,135 +2078,135 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Туризм</t>
+          <t>Новости</t>
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>112000</v>
+        <v>577</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>32000</v>
+        <v>350</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>4100</v>
+        <v>24</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>140</v>
+        <v>1</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>250</v>
+        <v>2</v>
       </c>
       <c r="J3" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K3" s="6" t="n">
-        <v>0.0401</v>
+        <v>0.04679999999999999</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>0.1403</v>
+        <v>0.0771</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Типичный Симферополь</t>
+          <t>Места Крыма</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>https://instagram.com/typical_simferopol</t>
+          <t>https://instagram.com/crimea.places</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Симферополь</t>
+          <t>Крым (Общий)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Общество</t>
+          <t>Туризм</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>43500</v>
+        <v>34200</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>8900</v>
+        <v>5200</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>1150</v>
+        <v>410</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>0.0289</v>
+        <v>0.0131</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>0.1412</v>
+        <v>0.0863</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Севастополь Life</t>
+          <t>Саша Лебедева | Фотограф</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>https://instagram.com/sevastopol_life</t>
+          <t>https://instagram.com/sasha.crimea</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Севастополь</t>
+          <t>Крым (Общий)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Общество</t>
+          <t>Культура</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>52100</v>
+        <v>12400</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>11200</v>
+        <v>2800</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>1540</v>
+        <v>380</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>90</v>
+        <v>18</v>
       </c>
       <c r="J5" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>0.03240000000000001</v>
+        <v>0.0331</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>0.1507</v>
+        <v>0.1464</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Ялта Life</t>
+          <t>Ялта Go</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>https://instagram.com/yalta_life</t>
+          <t>https://instagram.com/yalta.go</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -2216,124 +2216,170 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Общество</t>
+          <t>Туризм</t>
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>61200</v>
+        <v>28500</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>14500</v>
+        <v>2400</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>1920</v>
+        <v>210</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>74</v>
+        <v>7</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>125</v>
+        <v>12</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>0.0346</v>
+        <v>0.008</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>0.1461</v>
+        <v>0.09539999999999998</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Керчь Инфо</t>
+          <t>Севастополь Life</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>https://instagram.com/kerch_info</t>
+          <t>https://instagram.com/sevastopol.inst</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Керчь</t>
+          <t>Севастополь</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Новости</t>
+          <t>Общество</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>31400</v>
+        <v>21000</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>6200</v>
+        <v>3100</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>790</v>
+        <v>260</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>0.0274</v>
+        <v>0.0136</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>0.1389</v>
+        <v>0.09230000000000001</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Красивый Крым</t>
+          <t>Симферополь Крым</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>https://instagram.com/crimea_beauty</t>
+          <t>https://instagram.com/simferopol.crimea</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Крым (Общий)</t>
+          <t>Симферополь</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Туризм</t>
+          <t>Общество</t>
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>68400</v>
+        <v>8600</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>15600</v>
+        <v>1100</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>2200</v>
+        <v>95</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>80</v>
+        <v>3</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>180</v>
+        <v>6</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>0.036</v>
+        <v>0.0121</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>0.1577</v>
+        <v>0.09449999999999999</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Керчь Новости</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>https://instagram.com/kerch.news.inst</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Керчь</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Новости</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>4300</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>0.0153</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>0.08800000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -2350,8 +2396,8 @@
   <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
@@ -2429,12 +2475,12 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Вести Крым</t>
+          <t>Вести Крым (ОК)</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>https://ok.ru/vesticrimea</t>
+          <t>https://ok.ru/group/54508933054590</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -2448,39 +2494,39 @@
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>24500</v>
+        <v>16800</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>4800</v>
+        <v>2500</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>120</v>
+        <v>85</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K2" s="6" t="n">
-        <v>0.0073</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>0.0375</v>
+        <v>0.04679999999999999</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Крым 24</t>
+          <t>Крым 24 (ОК)</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>https://ok.ru/crimea24tv</t>
+          <t>https://ok.ru/tvcrimea24</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -2494,39 +2540,39 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>18200</v>
+        <v>13500</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>3500</v>
+        <v>2100</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="J3" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K3" s="6" t="n">
-        <v>0.0075</v>
+        <v>0.0073</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>0.0391</v>
+        <v>0.0467</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Типичный Симферополь</t>
+          <t>Типичный Симферополь (ОК)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>https://ok.ru/typical_simferopol</t>
+          <t>https://ok.ru/group/54316987416629</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -2540,28 +2586,28 @@
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>12500</v>
+        <v>9200</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>2100</v>
+        <v>1200</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="H4" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" s="5" t="n">
         <v>8</v>
-      </c>
-      <c r="I4" s="5" t="n">
-        <v>18</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>0.006500000000000001</v>
+        <v>0.0058</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>0.0386</v>
+        <v>0.0442</v>
       </c>
     </row>
   </sheetData>

</xml_diff>